<commit_message>
Ajout des terminologies officinales d3158e6f4bcaf133b49ed1cf90da9c095331650e
</commit_message>
<xml_diff>
--- a/nr-add-cip/ig/ValueSet-fr-medication-code.xlsx
+++ b/nr-add-cip/ig/ValueSet-fr-medication-code.xlsx
@@ -10,14 +10,12 @@
     <sheet name="Include #0" r:id="rId4" sheetId="2"/>
     <sheet name="Include #1" r:id="rId5" sheetId="3"/>
     <sheet name="Include #2" r:id="rId6" sheetId="4"/>
-    <sheet name="Include #3" r:id="rId7" sheetId="5"/>
-    <sheet name="Include #4" r:id="rId8" sheetId="6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
   <si>
     <t>Property</t>
   </si>
@@ -64,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-02T15:38:39+00:00</t>
+    <t>2026-02-02T15:38:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -125,9 +123,6 @@
   </si>
   <si>
     <t>http://data.esante.gouv.fr/ansm/medicament/substance</t>
-  </si>
-  <si>
-    <t>http://data.esante.gouv.fr/ansm/medicament/SpecialitePharmaceutique</t>
   </si>
 </sst>
 </file>
@@ -515,84 +510,4 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="30.703125" customWidth="true"/>
-    <col min="2" max="2" width="50.703125" customWidth="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="1">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s" s="2">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="30.703125" customWidth="true"/>
-    <col min="2" max="2" width="50.703125" customWidth="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="1">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s" s="2">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
 </file>
</xml_diff>